<commit_message>
feat(diagnostics): adiciona pré-mapeamento e mini-solver de reuniões de planejamento
</commit_message>
<xml_diff>
--- a/excel/GERADOR_DE_HORARIOS.xlsx
+++ b/excel/GERADOR_DE_HORARIOS.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\guilherme.odrumond\Projetos\GERADOR DE HORÁRIOS\excel\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{3B114353-EE53-486C-A003-AFE8F2C784D1}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{3DBA2249-8EA3-48D2-81BD-70164B8EE74F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" tabRatio="500" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" tabRatio="500" firstSheet="2" activeTab="3" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="CONFIG" sheetId="11" r:id="rId1"/>
@@ -34,6 +34,7 @@
     <definedName name="_xlnm._FilterDatabase" localSheetId="5" hidden="1">ATRIBUICOES!$A$1:$C$1037</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">DISPONIBILIDADE!$A$1:$AF$52</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="7" hidden="1">ESPECIALIDADES!$A$1:$G$46</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="4" hidden="1">PLANEJAMENTO!$A$1:$G$16</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="3" hidden="1">PROFESSORES!$A$1:$I$161</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">TURMAS!$A$1:$E$70</definedName>
   </definedNames>
@@ -58,7 +59,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="4965" uniqueCount="452">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="4981" uniqueCount="455">
   <si>
     <t>Turma</t>
   </si>
@@ -1414,6 +1415,15 @@
   </si>
   <si>
     <t>PROF BIOLOGIA 2</t>
+  </si>
+  <si>
+    <t>Grupo</t>
+  </si>
+  <si>
+    <t>A</t>
+  </si>
+  <si>
+    <t>B</t>
   </si>
 </sst>
 </file>
@@ -1673,7 +1683,7 @@
         <v>112</v>
       </c>
       <c r="B2" s="1">
-        <v>600</v>
+        <v>3600</v>
       </c>
     </row>
     <row r="3" spans="1:2" x14ac:dyDescent="0.25">
@@ -7643,7 +7653,7 @@
         <v>5</v>
       </c>
       <c r="H7" s="1">
-        <v>7</v>
+        <v>5</v>
       </c>
       <c r="I7" s="1" t="s">
         <v>129</v>
@@ -7991,7 +8001,7 @@
         <v>6</v>
       </c>
       <c r="H19" s="1">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="I19" s="1" t="s">
         <v>129</v>
@@ -9035,7 +9045,7 @@
         <v>5</v>
       </c>
       <c r="H55" s="1">
-        <v>7</v>
+        <v>5</v>
       </c>
       <c r="I55" s="1" t="s">
         <v>129</v>
@@ -9441,7 +9451,7 @@
         <v>5</v>
       </c>
       <c r="H69" s="1">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="I69" s="1" t="s">
         <v>129</v>
@@ -10456,7 +10466,7 @@
         <v>5</v>
       </c>
       <c r="H104" s="1">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="I104" s="1" t="s">
         <v>129</v>
@@ -10485,7 +10495,7 @@
         <v>4</v>
       </c>
       <c r="H105" s="1">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="I105" s="1" t="s">
         <v>129</v>
@@ -10775,7 +10785,7 @@
         <v>2</v>
       </c>
       <c r="H115" s="1">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="I115" s="1" t="s">
         <v>129</v>
@@ -10949,7 +10959,7 @@
         <v>5</v>
       </c>
       <c r="H121" s="1">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="I121" s="1" t="s">
         <v>129</v>
@@ -11152,7 +11162,7 @@
         <v>5</v>
       </c>
       <c r="H128" s="1">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="I128" s="1" t="s">
         <v>129</v>
@@ -11239,7 +11249,7 @@
         <v>6</v>
       </c>
       <c r="H131" s="1">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="I131" s="1" t="s">
         <v>129</v>
@@ -11558,7 +11568,7 @@
         <v>5</v>
       </c>
       <c r="H142" s="1">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="I142" s="1" t="s">
         <v>129</v>
@@ -11587,7 +11597,7 @@
         <v>8</v>
       </c>
       <c r="H143" s="1">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="I143" s="1" t="s">
         <v>129</v>
@@ -11848,7 +11858,7 @@
         <v>4</v>
       </c>
       <c r="H152" s="1">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="I152" s="1" t="s">
         <v>129</v>
@@ -11935,7 +11945,7 @@
         <v>5</v>
       </c>
       <c r="H155" s="1">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="I155" s="1" t="s">
         <v>129</v>
@@ -14022,7 +14032,7 @@
 
 <file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{AE4DB728-FCF3-4F70-830B-D6CC59807522}">
-  <dimension ref="A1:F16"/>
+  <dimension ref="A1:G16"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="25.42578125" customWidth="1"/>
@@ -14031,7 +14041,7 @@
     <col min="6" max="6" width="20" style="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A1" t="s">
         <v>254</v>
       </c>
@@ -14050,10 +14060,13 @@
       <c r="F1" s="1" t="s">
         <v>30</v>
       </c>
-    </row>
-    <row r="2" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="G1" s="1" t="s">
+        <v>452</v>
+      </c>
+    </row>
+    <row r="2" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
-        <v>436</v>
+        <v>439</v>
       </c>
       <c r="B2" s="1">
         <v>2</v>
@@ -14062,40 +14075,49 @@
         <v>1</v>
       </c>
       <c r="E2" s="1" t="s">
-        <v>46</v>
-      </c>
-    </row>
-    <row r="3" spans="1:6" x14ac:dyDescent="0.25">
+        <v>35</v>
+      </c>
+      <c r="G2" s="1" t="s">
+        <v>453</v>
+      </c>
+    </row>
+    <row r="3" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
-        <v>437</v>
+        <v>443</v>
       </c>
       <c r="B3" s="1">
         <v>2</v>
       </c>
       <c r="C3" s="1">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="E3" s="1" t="s">
-        <v>51</v>
-      </c>
-    </row>
-    <row r="4" spans="1:6" x14ac:dyDescent="0.25">
+        <v>35</v>
+      </c>
+      <c r="G3" s="1" t="s">
+        <v>453</v>
+      </c>
+    </row>
+    <row r="4" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
-        <v>438</v>
+        <v>447</v>
       </c>
       <c r="B4" s="1">
         <v>2</v>
       </c>
       <c r="C4" s="1">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="E4" s="1" t="s">
-        <v>40</v>
-      </c>
-    </row>
-    <row r="5" spans="1:6" x14ac:dyDescent="0.25">
+        <v>35</v>
+      </c>
+      <c r="G4" s="1" t="s">
+        <v>453</v>
+      </c>
+    </row>
+    <row r="5" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
-        <v>439</v>
+        <v>438</v>
       </c>
       <c r="B5" s="1">
         <v>2</v>
@@ -14104,44 +14126,47 @@
         <v>1</v>
       </c>
       <c r="E5" s="1" t="s">
-        <v>35</v>
-      </c>
-    </row>
-    <row r="6" spans="1:6" x14ac:dyDescent="0.25">
+        <v>40</v>
+      </c>
+      <c r="G5" s="1" t="s">
+        <v>453</v>
+      </c>
+    </row>
+    <row r="6" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A6" t="s">
-        <v>398</v>
+        <v>442</v>
       </c>
       <c r="B6" s="1">
         <v>2</v>
       </c>
-      <c r="C6" s="1" t="s">
-        <v>256</v>
-      </c>
-      <c r="D6" s="1" t="s">
-        <v>110</v>
+      <c r="C6" s="1">
+        <v>2</v>
       </c>
       <c r="E6" s="1" t="s">
-        <v>43</v>
-      </c>
-    </row>
-    <row r="7" spans="1:6" x14ac:dyDescent="0.25">
+        <v>40</v>
+      </c>
+      <c r="G6" s="1" t="s">
+        <v>453</v>
+      </c>
+    </row>
+    <row r="7" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A7" t="s">
-        <v>399</v>
+        <v>446</v>
       </c>
       <c r="B7" s="1">
         <v>2</v>
       </c>
-      <c r="C7" s="1" t="s">
-        <v>256</v>
-      </c>
-      <c r="D7" s="1" t="s">
-        <v>397</v>
+      <c r="C7" s="1">
+        <v>3</v>
       </c>
       <c r="E7" s="1" t="s">
-        <v>43</v>
-      </c>
-    </row>
-    <row r="8" spans="1:6" x14ac:dyDescent="0.25">
+        <v>40</v>
+      </c>
+      <c r="G7" s="1" t="s">
+        <v>453</v>
+      </c>
+    </row>
+    <row r="8" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A8" t="s">
         <v>400</v>
       </c>
@@ -14157,52 +14182,70 @@
       <c r="E8" s="1" t="s">
         <v>43</v>
       </c>
-    </row>
-    <row r="9" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="G8" s="1" t="s">
+        <v>453</v>
+      </c>
+    </row>
+    <row r="9" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A9" t="s">
-        <v>440</v>
+        <v>399</v>
       </c>
       <c r="B9" s="1">
         <v>2</v>
       </c>
-      <c r="C9" s="1">
-        <v>2</v>
+      <c r="C9" s="1" t="s">
+        <v>256</v>
+      </c>
+      <c r="D9" s="1" t="s">
+        <v>397</v>
       </c>
       <c r="E9" s="1" t="s">
-        <v>46</v>
-      </c>
-    </row>
-    <row r="10" spans="1:6" x14ac:dyDescent="0.25">
+        <v>43</v>
+      </c>
+      <c r="G9" s="1" t="s">
+        <v>453</v>
+      </c>
+    </row>
+    <row r="10" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A10" t="s">
-        <v>441</v>
+        <v>398</v>
       </c>
       <c r="B10" s="1">
         <v>2</v>
       </c>
-      <c r="C10" s="1">
-        <v>2</v>
+      <c r="C10" s="1" t="s">
+        <v>256</v>
+      </c>
+      <c r="D10" s="1" t="s">
+        <v>110</v>
       </c>
       <c r="E10" s="1" t="s">
-        <v>51</v>
-      </c>
-    </row>
-    <row r="11" spans="1:6" x14ac:dyDescent="0.25">
+        <v>43</v>
+      </c>
+      <c r="G10" s="1" t="s">
+        <v>454</v>
+      </c>
+    </row>
+    <row r="11" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A11" t="s">
-        <v>442</v>
+        <v>436</v>
       </c>
       <c r="B11" s="1">
         <v>2</v>
       </c>
       <c r="C11" s="1">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="E11" s="1" t="s">
-        <v>40</v>
-      </c>
-    </row>
-    <row r="12" spans="1:6" x14ac:dyDescent="0.25">
+        <v>46</v>
+      </c>
+      <c r="G11" s="1" t="s">
+        <v>454</v>
+      </c>
+    </row>
+    <row r="12" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A12" t="s">
-        <v>443</v>
+        <v>440</v>
       </c>
       <c r="B12" s="1">
         <v>2</v>
@@ -14211,10 +14254,13 @@
         <v>2</v>
       </c>
       <c r="E12" s="1" t="s">
-        <v>35</v>
-      </c>
-    </row>
-    <row r="13" spans="1:6" x14ac:dyDescent="0.25">
+        <v>46</v>
+      </c>
+      <c r="G12" s="1" t="s">
+        <v>454</v>
+      </c>
+    </row>
+    <row r="13" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A13" t="s">
         <v>444</v>
       </c>
@@ -14227,38 +14273,47 @@
       <c r="E13" s="1" t="s">
         <v>46</v>
       </c>
-    </row>
-    <row r="14" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="G13" s="1" t="s">
+        <v>454</v>
+      </c>
+    </row>
+    <row r="14" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A14" t="s">
-        <v>445</v>
+        <v>437</v>
       </c>
       <c r="B14" s="1">
         <v>2</v>
       </c>
       <c r="C14" s="1">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="E14" s="1" t="s">
         <v>51</v>
       </c>
-    </row>
-    <row r="15" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="G14" s="1" t="s">
+        <v>454</v>
+      </c>
+    </row>
+    <row r="15" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A15" t="s">
-        <v>446</v>
+        <v>441</v>
       </c>
       <c r="B15" s="1">
         <v>2</v>
       </c>
       <c r="C15" s="1">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="E15" s="1" t="s">
-        <v>40</v>
-      </c>
-    </row>
-    <row r="16" spans="1:6" x14ac:dyDescent="0.25">
+        <v>51</v>
+      </c>
+      <c r="G15" s="1" t="s">
+        <v>454</v>
+      </c>
+    </row>
+    <row r="16" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A16" t="s">
-        <v>447</v>
+        <v>445</v>
       </c>
       <c r="B16" s="1">
         <v>2</v>
@@ -14267,15 +14322,20 @@
         <v>3</v>
       </c>
       <c r="E16" s="1" t="s">
-        <v>35</v>
+        <v>51</v>
+      </c>
+      <c r="G16" s="1" t="s">
+        <v>454</v>
       </c>
     </row>
   </sheetData>
+  <autoFilter ref="A1:G16" xr:uid="{AE4DB728-FCF3-4F70-830B-D6CC59807522}">
+    <sortState xmlns:xlrd2="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata2" ref="A2:G16">
+      <sortCondition ref="A1:A16"/>
+    </sortState>
+  </autoFilter>
   <phoneticPr fontId="1" type="noConversion"/>
   <pageMargins left="0.511811024" right="0.511811024" top="0.78740157499999996" bottom="0.78740157499999996" header="0.31496062000000002" footer="0.31496062000000002"/>
-  <ignoredErrors>
-    <ignoredError sqref="C6 C7:C8" twoDigitTextYear="1"/>
-  </ignoredErrors>
   <extLst>
     <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{CCE6A557-97BC-4b89-ADB6-D9C93CAAB3DF}">
       <x14:dataValidations xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main" count="1">

</xml_diff>

<commit_message>
feat(horario): fecha modelo completo com Max Dias rígido após ajuste de 5 professores
</commit_message>
<xml_diff>
--- a/excel/GERADOR_DE_HORARIOS.xlsx
+++ b/excel/GERADOR_DE_HORARIOS.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\guilherme.odrumond\Projetos\GERADOR DE HORÁRIOS\excel\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{3C7B26CC-AD63-4461-8121-B1F0E9F40FF7}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{344EEEA2-39D6-4600-BC32-4A9E33A8D2D7}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" tabRatio="500" activeTab="4" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" tabRatio="500" activeTab="3" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="CONFIG" sheetId="11" r:id="rId1"/>
@@ -32,7 +32,7 @@
   </sheets>
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="5" hidden="1">ATRIBUICOES!$A$1:$C$1037</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">DISPONIBILIDADE!$A$1:$AF$52</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">DISPONIBILIDADE!$A$1:$AF$33</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="7" hidden="1">ESPECIALIDADES!$A$1:$G$46</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="4" hidden="1">PLANEJAMENTO!$A$1:$G$16</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="3" hidden="1">PROFESSORES!$A$1:$I$161</definedName>
@@ -59,7 +59,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="4966" uniqueCount="453">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="4935" uniqueCount="453">
   <si>
     <t>Turma</t>
   </si>
@@ -1424,7 +1424,7 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="2" x14ac:knownFonts="1">
+  <fonts count="3" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -1437,6 +1437,13 @@
       <name val="Aptos Narrow"/>
       <family val="2"/>
       <charset val="1"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="11"/>
+      <color rgb="FFFF0000"/>
+      <name val="Aptos Narrow"/>
+      <family val="2"/>
     </font>
   </fonts>
   <fills count="2">
@@ -1459,9 +1466,12 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="2">
+  <cellXfs count="3">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
   </cellXfs>
@@ -2878,7 +2888,7 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{59A23CC3-1A6A-46FD-BA52-7A9B0C051B2C}">
-  <dimension ref="A1:AF45"/>
+  <dimension ref="A1:AF26"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="22.140625" bestFit="1" customWidth="1"/>
@@ -2983,254 +2993,317 @@
     </row>
     <row r="2" spans="1:32" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
-        <v>261</v>
+        <v>264</v>
       </c>
       <c r="B2" s="1">
-        <f>COUNTBLANK(C2:AF2)</f>
+        <f t="shared" ref="B2:B26" si="0">COUNTBLANK(C2:AF2)</f>
         <v>24</v>
       </c>
-      <c r="O2" s="1" t="s">
+      <c r="AA2" s="1" t="s">
         <v>398</v>
       </c>
-      <c r="P2" s="1" t="s">
+      <c r="AB2" s="1" t="s">
         <v>398</v>
       </c>
-      <c r="Q2" s="1" t="s">
+      <c r="AC2" s="1" t="s">
         <v>398</v>
       </c>
-      <c r="R2" s="1" t="s">
+      <c r="AD2" s="1" t="s">
         <v>398</v>
       </c>
-      <c r="S2" s="1" t="s">
+      <c r="AE2" s="1" t="s">
         <v>398</v>
       </c>
-      <c r="T2" s="1" t="s">
+      <c r="AF2" s="1" t="s">
         <v>398</v>
       </c>
     </row>
     <row r="3" spans="1:32" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
-        <v>264</v>
+        <v>268</v>
       </c>
       <c r="B3" s="1">
-        <f t="shared" ref="B3:B45" si="0">COUNTBLANK(C3:AF3)</f>
-        <v>24</v>
-      </c>
-      <c r="AA3" s="1" t="s">
+        <f t="shared" si="0"/>
+        <v>26</v>
+      </c>
+      <c r="O3" s="1" t="s">
         <v>398</v>
       </c>
-      <c r="AB3" s="1" t="s">
+      <c r="P3" s="1" t="s">
         <v>398</v>
       </c>
-      <c r="AC3" s="1" t="s">
+      <c r="Q3" s="1" t="s">
         <v>398</v>
       </c>
-      <c r="AD3" s="1" t="s">
-        <v>398</v>
-      </c>
-      <c r="AE3" s="1" t="s">
-        <v>398</v>
-      </c>
-      <c r="AF3" s="1" t="s">
+      <c r="R3" s="1" t="s">
         <v>398</v>
       </c>
     </row>
     <row r="4" spans="1:32" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
-        <v>268</v>
+        <v>263</v>
       </c>
       <c r="B4" s="1">
         <f t="shared" si="0"/>
-        <v>26</v>
-      </c>
-      <c r="O4" s="1" t="s">
-        <v>398</v>
-      </c>
-      <c r="P4" s="1" t="s">
-        <v>398</v>
-      </c>
-      <c r="Q4" s="1" t="s">
-        <v>398</v>
-      </c>
-      <c r="R4" s="1" t="s">
+        <v>29</v>
+      </c>
+      <c r="T4" s="1" t="s">
         <v>398</v>
       </c>
     </row>
     <row r="5" spans="1:32" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
-        <v>263</v>
+        <v>273</v>
       </c>
       <c r="B5" s="1">
         <f t="shared" si="0"/>
-        <v>29</v>
-      </c>
-      <c r="T5" s="1" t="s">
+        <v>24</v>
+      </c>
+      <c r="I5" s="1" t="s">
+        <v>398</v>
+      </c>
+      <c r="J5" s="1" t="s">
+        <v>398</v>
+      </c>
+      <c r="K5" s="1" t="s">
+        <v>398</v>
+      </c>
+      <c r="L5" s="1" t="s">
+        <v>398</v>
+      </c>
+      <c r="M5" s="1" t="s">
+        <v>398</v>
+      </c>
+      <c r="N5" s="1" t="s">
         <v>398</v>
       </c>
     </row>
     <row r="6" spans="1:32" x14ac:dyDescent="0.25">
       <c r="A6" t="s">
-        <v>271</v>
+        <v>275</v>
       </c>
       <c r="B6" s="1">
         <f t="shared" si="0"/>
-        <v>30</v>
+        <v>26</v>
+      </c>
+      <c r="U6" s="1" t="s">
+        <v>398</v>
+      </c>
+      <c r="V6" s="1" t="s">
+        <v>398</v>
+      </c>
+      <c r="W6" s="1" t="s">
+        <v>398</v>
+      </c>
+      <c r="X6" s="1" t="s">
+        <v>398</v>
       </c>
     </row>
     <row r="7" spans="1:32" x14ac:dyDescent="0.25">
       <c r="A7" t="s">
-        <v>273</v>
+        <v>286</v>
       </c>
       <c r="B7" s="1">
         <f t="shared" si="0"/>
-        <v>24</v>
+        <v>26</v>
+      </c>
+      <c r="C7" s="1" t="s">
+        <v>431</v>
       </c>
       <c r="I7" s="1" t="s">
-        <v>398</v>
-      </c>
-      <c r="J7" s="1" t="s">
-        <v>398</v>
-      </c>
-      <c r="K7" s="1" t="s">
-        <v>398</v>
-      </c>
-      <c r="L7" s="1" t="s">
-        <v>398</v>
-      </c>
-      <c r="M7" s="1" t="s">
-        <v>398</v>
-      </c>
-      <c r="N7" s="1" t="s">
-        <v>398</v>
+        <v>431</v>
+      </c>
+      <c r="O7" s="1" t="s">
+        <v>431</v>
+      </c>
+      <c r="AA7" s="1" t="s">
+        <v>431</v>
       </c>
     </row>
     <row r="8" spans="1:32" x14ac:dyDescent="0.25">
       <c r="A8" t="s">
-        <v>275</v>
+        <v>303</v>
       </c>
       <c r="B8" s="1">
         <f t="shared" si="0"/>
-        <v>26</v>
-      </c>
-      <c r="U8" s="1" t="s">
+        <v>28</v>
+      </c>
+      <c r="C8" s="1" t="s">
         <v>398</v>
       </c>
-      <c r="V8" s="1" t="s">
-        <v>398</v>
-      </c>
-      <c r="W8" s="1" t="s">
-        <v>398</v>
-      </c>
-      <c r="X8" s="1" t="s">
+      <c r="D8" s="1" t="s">
         <v>398</v>
       </c>
     </row>
     <row r="9" spans="1:32" x14ac:dyDescent="0.25">
       <c r="A9" t="s">
-        <v>276</v>
+        <v>317</v>
       </c>
       <c r="B9" s="1">
         <f t="shared" si="0"/>
-        <v>30</v>
+        <v>24</v>
+      </c>
+      <c r="U9" s="1" t="s">
+        <v>431</v>
+      </c>
+      <c r="V9" s="1" t="s">
+        <v>431</v>
+      </c>
+      <c r="W9" s="1" t="s">
+        <v>431</v>
+      </c>
+      <c r="X9" s="1" t="s">
+        <v>431</v>
+      </c>
+      <c r="Y9" s="1" t="s">
+        <v>431</v>
+      </c>
+      <c r="Z9" s="1" t="s">
+        <v>431</v>
       </c>
     </row>
     <row r="10" spans="1:32" x14ac:dyDescent="0.25">
       <c r="A10" t="s">
-        <v>283</v>
+        <v>319</v>
       </c>
       <c r="B10" s="1">
         <f t="shared" si="0"/>
-        <v>30</v>
+        <v>28</v>
+      </c>
+      <c r="AE10" s="1" t="s">
+        <v>398</v>
+      </c>
+      <c r="AF10" s="1" t="s">
+        <v>398</v>
       </c>
     </row>
     <row r="11" spans="1:32" x14ac:dyDescent="0.25">
       <c r="A11" t="s">
-        <v>286</v>
+        <v>324</v>
       </c>
       <c r="B11" s="1">
         <f t="shared" si="0"/>
-        <v>26</v>
-      </c>
-      <c r="C11" s="1" t="s">
-        <v>431</v>
-      </c>
-      <c r="I11" s="1" t="s">
-        <v>431</v>
-      </c>
-      <c r="O11" s="1" t="s">
-        <v>431</v>
-      </c>
-      <c r="AA11" s="1" t="s">
-        <v>431</v>
+        <v>28</v>
+      </c>
+      <c r="AE11" s="1" t="s">
+        <v>398</v>
+      </c>
+      <c r="AF11" s="1" t="s">
+        <v>398</v>
       </c>
     </row>
     <row r="12" spans="1:32" x14ac:dyDescent="0.25">
       <c r="A12" t="s">
-        <v>289</v>
+        <v>328</v>
       </c>
       <c r="B12" s="1">
         <f t="shared" si="0"/>
-        <v>30</v>
+        <v>26</v>
+      </c>
+      <c r="I12" s="1" t="s">
+        <v>398</v>
+      </c>
+      <c r="J12" s="1" t="s">
+        <v>398</v>
+      </c>
+      <c r="O12" s="1" t="s">
+        <v>398</v>
+      </c>
+      <c r="P12" s="1" t="s">
+        <v>398</v>
       </c>
     </row>
     <row r="13" spans="1:32" x14ac:dyDescent="0.25">
       <c r="A13" t="s">
-        <v>303</v>
+        <v>331</v>
       </c>
       <c r="B13" s="1">
         <f t="shared" si="0"/>
-        <v>28</v>
-      </c>
-      <c r="C13" s="1" t="s">
+        <v>27</v>
+      </c>
+      <c r="O13" s="1" t="s">
         <v>398</v>
       </c>
-      <c r="D13" s="1" t="s">
+      <c r="U13" s="1" t="s">
+        <v>398</v>
+      </c>
+      <c r="AA13" s="1" t="s">
         <v>398</v>
       </c>
     </row>
     <row r="14" spans="1:32" x14ac:dyDescent="0.25">
       <c r="A14" t="s">
-        <v>305</v>
+        <v>336</v>
       </c>
       <c r="B14" s="1">
         <f t="shared" si="0"/>
-        <v>30</v>
+        <v>24</v>
+      </c>
+      <c r="C14" s="1" t="s">
+        <v>398</v>
+      </c>
+      <c r="D14" s="1" t="s">
+        <v>398</v>
+      </c>
+      <c r="E14" s="1" t="s">
+        <v>398</v>
+      </c>
+      <c r="F14" s="1" t="s">
+        <v>398</v>
+      </c>
+      <c r="G14" s="1" t="s">
+        <v>398</v>
+      </c>
+      <c r="H14" s="1" t="s">
+        <v>398</v>
       </c>
     </row>
     <row r="15" spans="1:32" x14ac:dyDescent="0.25">
       <c r="A15" t="s">
-        <v>317</v>
+        <v>337</v>
       </c>
       <c r="B15" s="1">
         <f t="shared" si="0"/>
-        <v>24</v>
-      </c>
-      <c r="U15" s="1" t="s">
-        <v>431</v>
-      </c>
-      <c r="V15" s="1" t="s">
-        <v>431</v>
-      </c>
-      <c r="W15" s="1" t="s">
-        <v>431</v>
-      </c>
-      <c r="X15" s="1" t="s">
-        <v>431</v>
-      </c>
-      <c r="Y15" s="1" t="s">
-        <v>431</v>
-      </c>
-      <c r="Z15" s="1" t="s">
-        <v>431</v>
+        <v>26</v>
+      </c>
+      <c r="O15" s="1" t="s">
+        <v>398</v>
+      </c>
+      <c r="P15" s="1" t="s">
+        <v>398</v>
+      </c>
+      <c r="Q15" s="1" t="s">
+        <v>398</v>
+      </c>
+      <c r="R15" s="1" t="s">
+        <v>398</v>
       </c>
     </row>
     <row r="16" spans="1:32" x14ac:dyDescent="0.25">
       <c r="A16" t="s">
-        <v>319</v>
+        <v>340</v>
       </c>
       <c r="B16" s="1">
         <f t="shared" si="0"/>
-        <v>28</v>
+        <v>22</v>
+      </c>
+      <c r="G16" s="1" t="s">
+        <v>398</v>
+      </c>
+      <c r="H16" s="1" t="s">
+        <v>398</v>
+      </c>
+      <c r="M16" s="1" t="s">
+        <v>398</v>
+      </c>
+      <c r="N16" s="1" t="s">
+        <v>398</v>
+      </c>
+      <c r="S16" s="1" t="s">
+        <v>398</v>
+      </c>
+      <c r="T16" s="1" t="s">
+        <v>398</v>
       </c>
       <c r="AE16" s="1" t="s">
         <v>398</v>
@@ -3241,152 +3314,194 @@
     </row>
     <row r="17" spans="1:32" x14ac:dyDescent="0.25">
       <c r="A17" t="s">
-        <v>324</v>
+        <v>347</v>
       </c>
       <c r="B17" s="1">
         <f t="shared" si="0"/>
         <v>28</v>
       </c>
-      <c r="AE17" s="1" t="s">
+      <c r="C17" s="1" t="s">
         <v>398</v>
       </c>
-      <c r="AF17" s="1" t="s">
+      <c r="D17" s="1" t="s">
         <v>398</v>
       </c>
     </row>
     <row r="18" spans="1:32" x14ac:dyDescent="0.25">
       <c r="A18" t="s">
-        <v>325</v>
+        <v>355</v>
       </c>
       <c r="B18" s="1">
         <f t="shared" si="0"/>
-        <v>30</v>
+        <v>26</v>
+      </c>
+      <c r="M18" s="1" t="s">
+        <v>431</v>
+      </c>
+      <c r="N18" s="1" t="s">
+        <v>431</v>
+      </c>
+      <c r="Y18" s="1" t="s">
+        <v>431</v>
+      </c>
+      <c r="Z18" s="1" t="s">
+        <v>431</v>
       </c>
     </row>
     <row r="19" spans="1:32" x14ac:dyDescent="0.25">
       <c r="A19" t="s">
-        <v>327</v>
+        <v>362</v>
       </c>
       <c r="B19" s="1">
         <f t="shared" si="0"/>
-        <v>30</v>
+        <v>27</v>
+      </c>
+      <c r="R19" s="1" t="s">
+        <v>431</v>
+      </c>
+      <c r="S19" s="1" t="s">
+        <v>431</v>
+      </c>
+      <c r="T19" s="1" t="s">
+        <v>431</v>
       </c>
     </row>
     <row r="20" spans="1:32" x14ac:dyDescent="0.25">
       <c r="A20" t="s">
-        <v>328</v>
+        <v>369</v>
       </c>
       <c r="B20" s="1">
         <f t="shared" si="0"/>
-        <v>26</v>
+        <v>23</v>
       </c>
       <c r="I20" s="1" t="s">
-        <v>398</v>
+        <v>431</v>
       </c>
       <c r="J20" s="1" t="s">
-        <v>398</v>
+        <v>431</v>
+      </c>
+      <c r="K20" s="1" t="s">
+        <v>431</v>
       </c>
       <c r="O20" s="1" t="s">
-        <v>398</v>
+        <v>431</v>
       </c>
       <c r="P20" s="1" t="s">
-        <v>398</v>
+        <v>431</v>
+      </c>
+      <c r="Q20" s="1" t="s">
+        <v>431</v>
+      </c>
+      <c r="R20" s="1" t="s">
+        <v>431</v>
       </c>
     </row>
     <row r="21" spans="1:32" x14ac:dyDescent="0.25">
       <c r="A21" t="s">
-        <v>330</v>
+        <v>371</v>
       </c>
       <c r="B21" s="1">
         <f t="shared" si="0"/>
-        <v>30</v>
+        <v>24</v>
+      </c>
+      <c r="C21" s="1" t="s">
+        <v>431</v>
+      </c>
+      <c r="D21" s="1" t="s">
+        <v>431</v>
+      </c>
+      <c r="E21" s="1" t="s">
+        <v>431</v>
+      </c>
+      <c r="F21" s="1" t="s">
+        <v>431</v>
+      </c>
+      <c r="G21" s="1" t="s">
+        <v>431</v>
+      </c>
+      <c r="H21" s="1" t="s">
+        <v>431</v>
       </c>
     </row>
     <row r="22" spans="1:32" x14ac:dyDescent="0.25">
       <c r="A22" t="s">
-        <v>331</v>
+        <v>379</v>
       </c>
       <c r="B22" s="1">
         <f t="shared" si="0"/>
-        <v>27</v>
-      </c>
-      <c r="O22" s="1" t="s">
-        <v>398</v>
-      </c>
-      <c r="U22" s="1" t="s">
-        <v>398</v>
-      </c>
-      <c r="AA22" s="1" t="s">
-        <v>398</v>
+        <v>24</v>
+      </c>
+      <c r="H22" s="1" t="s">
+        <v>431</v>
+      </c>
+      <c r="N22" s="1" t="s">
+        <v>431</v>
+      </c>
+      <c r="T22" s="1" t="s">
+        <v>431</v>
+      </c>
+      <c r="Z22" s="1" t="s">
+        <v>431</v>
+      </c>
+      <c r="AE22" s="1" t="s">
+        <v>431</v>
+      </c>
+      <c r="AF22" s="1" t="s">
+        <v>431</v>
       </c>
     </row>
     <row r="23" spans="1:32" x14ac:dyDescent="0.25">
       <c r="A23" t="s">
-        <v>336</v>
+        <v>383</v>
       </c>
       <c r="B23" s="1">
         <f t="shared" si="0"/>
-        <v>24</v>
-      </c>
-      <c r="C23" s="1" t="s">
-        <v>398</v>
-      </c>
-      <c r="D23" s="1" t="s">
-        <v>398</v>
-      </c>
-      <c r="E23" s="1" t="s">
-        <v>398</v>
-      </c>
-      <c r="F23" s="1" t="s">
-        <v>398</v>
-      </c>
-      <c r="G23" s="1" t="s">
-        <v>398</v>
-      </c>
-      <c r="H23" s="1" t="s">
-        <v>398</v>
+        <v>27</v>
+      </c>
+      <c r="N23" s="1" t="s">
+        <v>431</v>
+      </c>
+      <c r="AE23" s="1" t="s">
+        <v>431</v>
+      </c>
+      <c r="AF23" s="1" t="s">
+        <v>431</v>
       </c>
     </row>
     <row r="24" spans="1:32" x14ac:dyDescent="0.25">
       <c r="A24" t="s">
-        <v>337</v>
+        <v>390</v>
       </c>
       <c r="B24" s="1">
         <f t="shared" si="0"/>
-        <v>26</v>
+        <v>24</v>
+      </c>
+      <c r="M24" s="1" t="s">
+        <v>431</v>
+      </c>
+      <c r="N24" s="1" t="s">
+        <v>431</v>
       </c>
       <c r="O24" s="1" t="s">
-        <v>398</v>
-      </c>
-      <c r="P24" s="1" t="s">
-        <v>398</v>
-      </c>
-      <c r="Q24" s="1" t="s">
-        <v>398</v>
-      </c>
-      <c r="R24" s="1" t="s">
-        <v>398</v>
+        <v>431</v>
+      </c>
+      <c r="U24" s="1" t="s">
+        <v>431</v>
+      </c>
+      <c r="AE24" s="1" t="s">
+        <v>431</v>
+      </c>
+      <c r="AF24" s="1" t="s">
+        <v>431</v>
       </c>
     </row>
     <row r="25" spans="1:32" x14ac:dyDescent="0.25">
       <c r="A25" t="s">
-        <v>340</v>
+        <v>381</v>
       </c>
       <c r="B25" s="1">
         <f t="shared" si="0"/>
-        <v>22</v>
-      </c>
-      <c r="G25" s="1" t="s">
-        <v>398</v>
-      </c>
-      <c r="H25" s="1" t="s">
-        <v>398</v>
-      </c>
-      <c r="M25" s="1" t="s">
-        <v>398</v>
-      </c>
-      <c r="N25" s="1" t="s">
-        <v>398</v>
+        <v>28</v>
       </c>
       <c r="S25" s="1" t="s">
         <v>398</v>
@@ -3394,349 +3509,32 @@
       <c r="T25" s="1" t="s">
         <v>398</v>
       </c>
-      <c r="AE25" s="1" t="s">
-        <v>398</v>
-      </c>
-      <c r="AF25" s="1" t="s">
-        <v>398</v>
-      </c>
     </row>
     <row r="26" spans="1:32" x14ac:dyDescent="0.25">
       <c r="A26" t="s">
-        <v>343</v>
+        <v>281</v>
       </c>
       <c r="B26" s="1">
         <f t="shared" si="0"/>
-        <v>30</v>
-      </c>
-    </row>
-    <row r="27" spans="1:32" x14ac:dyDescent="0.25">
-      <c r="A27" t="s">
-        <v>347</v>
-      </c>
-      <c r="B27" s="1">
-        <f t="shared" si="0"/>
-        <v>28</v>
-      </c>
-      <c r="C27" s="1" t="s">
+        <v>25</v>
+      </c>
+      <c r="H26" s="1" t="s">
         <v>398</v>
       </c>
-      <c r="D27" s="1" t="s">
+      <c r="N26" s="1" t="s">
         <v>398</v>
       </c>
-    </row>
-    <row r="28" spans="1:32" x14ac:dyDescent="0.25">
-      <c r="A28" t="s">
-        <v>350</v>
-      </c>
-      <c r="B28" s="1">
-        <f t="shared" si="0"/>
-        <v>30</v>
-      </c>
-    </row>
-    <row r="29" spans="1:32" x14ac:dyDescent="0.25">
-      <c r="A29" t="s">
-        <v>352</v>
-      </c>
-      <c r="B29" s="1">
-        <f t="shared" si="0"/>
-        <v>30</v>
-      </c>
-    </row>
-    <row r="30" spans="1:32" x14ac:dyDescent="0.25">
-      <c r="A30" t="s">
-        <v>416</v>
-      </c>
-      <c r="B30" s="1">
-        <f t="shared" si="0"/>
-        <v>30</v>
-      </c>
-    </row>
-    <row r="31" spans="1:32" x14ac:dyDescent="0.25">
-      <c r="A31" t="s">
-        <v>355</v>
-      </c>
-      <c r="B31" s="1">
-        <f t="shared" si="0"/>
-        <v>26</v>
-      </c>
-      <c r="M31" s="1" t="s">
-        <v>431</v>
-      </c>
-      <c r="N31" s="1" t="s">
-        <v>431</v>
-      </c>
-      <c r="Y31" s="1" t="s">
-        <v>431</v>
-      </c>
-      <c r="Z31" s="1" t="s">
-        <v>431</v>
-      </c>
-    </row>
-    <row r="32" spans="1:32" x14ac:dyDescent="0.25">
-      <c r="A32" t="s">
-        <v>358</v>
-      </c>
-      <c r="B32" s="1">
-        <f t="shared" si="0"/>
-        <v>24</v>
-      </c>
-      <c r="AA32" s="1" t="s">
-        <v>431</v>
-      </c>
-      <c r="AB32" s="1" t="s">
-        <v>431</v>
-      </c>
-      <c r="AC32" s="1" t="s">
-        <v>431</v>
-      </c>
-      <c r="AD32" s="1" t="s">
-        <v>431</v>
-      </c>
-      <c r="AE32" s="1" t="s">
-        <v>431</v>
-      </c>
-      <c r="AF32" s="1" t="s">
-        <v>431</v>
-      </c>
-    </row>
-    <row r="33" spans="1:32" x14ac:dyDescent="0.25">
-      <c r="A33" t="s">
-        <v>361</v>
-      </c>
-      <c r="B33" s="1">
-        <f t="shared" si="0"/>
-        <v>30</v>
-      </c>
-    </row>
-    <row r="34" spans="1:32" x14ac:dyDescent="0.25">
-      <c r="A34" t="s">
-        <v>362</v>
-      </c>
-      <c r="B34" s="1">
-        <f t="shared" si="0"/>
-        <v>27</v>
-      </c>
-      <c r="R34" s="1" t="s">
-        <v>431</v>
-      </c>
-      <c r="S34" s="1" t="s">
-        <v>431</v>
-      </c>
-      <c r="T34" s="1" t="s">
-        <v>431</v>
-      </c>
-    </row>
-    <row r="35" spans="1:32" x14ac:dyDescent="0.25">
-      <c r="A35" t="s">
-        <v>369</v>
-      </c>
-      <c r="B35" s="1">
-        <f t="shared" si="0"/>
-        <v>23</v>
-      </c>
-      <c r="I35" s="1" t="s">
-        <v>431</v>
-      </c>
-      <c r="J35" s="1" t="s">
-        <v>431</v>
-      </c>
-      <c r="K35" s="1" t="s">
-        <v>431</v>
-      </c>
-      <c r="O35" s="1" t="s">
-        <v>431</v>
-      </c>
-      <c r="P35" s="1" t="s">
-        <v>431</v>
-      </c>
-      <c r="Q35" s="1" t="s">
-        <v>431</v>
-      </c>
-      <c r="R35" s="1" t="s">
-        <v>431</v>
-      </c>
-    </row>
-    <row r="36" spans="1:32" x14ac:dyDescent="0.25">
-      <c r="A36" t="s">
-        <v>371</v>
-      </c>
-      <c r="B36" s="1">
-        <f t="shared" si="0"/>
-        <v>24</v>
-      </c>
-      <c r="C36" s="1" t="s">
-        <v>431</v>
-      </c>
-      <c r="D36" s="1" t="s">
-        <v>431</v>
-      </c>
-      <c r="E36" s="1" t="s">
-        <v>431</v>
-      </c>
-      <c r="F36" s="1" t="s">
-        <v>431</v>
-      </c>
-      <c r="G36" s="1" t="s">
-        <v>431</v>
-      </c>
-      <c r="H36" s="1" t="s">
-        <v>431</v>
-      </c>
-    </row>
-    <row r="37" spans="1:32" x14ac:dyDescent="0.25">
-      <c r="A37" t="s">
-        <v>372</v>
-      </c>
-      <c r="B37" s="1">
-        <f t="shared" si="0"/>
-        <v>30</v>
-      </c>
-    </row>
-    <row r="38" spans="1:32" x14ac:dyDescent="0.25">
-      <c r="A38" t="s">
-        <v>379</v>
-      </c>
-      <c r="B38" s="1">
-        <f t="shared" si="0"/>
-        <v>24</v>
-      </c>
-      <c r="H38" s="1" t="s">
-        <v>431</v>
-      </c>
-      <c r="N38" s="1" t="s">
-        <v>431</v>
-      </c>
-      <c r="T38" s="1" t="s">
-        <v>431</v>
-      </c>
-      <c r="Z38" s="1" t="s">
-        <v>431</v>
-      </c>
-      <c r="AE38" s="1" t="s">
-        <v>431</v>
-      </c>
-      <c r="AF38" s="1" t="s">
-        <v>431</v>
-      </c>
-    </row>
-    <row r="39" spans="1:32" x14ac:dyDescent="0.25">
-      <c r="A39" t="s">
-        <v>383</v>
-      </c>
-      <c r="B39" s="1">
-        <f t="shared" si="0"/>
-        <v>27</v>
-      </c>
-      <c r="N39" s="1" t="s">
-        <v>431</v>
-      </c>
-      <c r="AE39" s="1" t="s">
-        <v>431</v>
-      </c>
-      <c r="AF39" s="1" t="s">
-        <v>431</v>
-      </c>
-    </row>
-    <row r="40" spans="1:32" x14ac:dyDescent="0.25">
-      <c r="A40" t="s">
-        <v>390</v>
-      </c>
-      <c r="B40" s="1">
-        <f t="shared" si="0"/>
-        <v>24</v>
-      </c>
-      <c r="M40" s="1" t="s">
-        <v>431</v>
-      </c>
-      <c r="N40" s="1" t="s">
-        <v>431</v>
-      </c>
-      <c r="O40" s="1" t="s">
-        <v>431</v>
-      </c>
-      <c r="U40" s="1" t="s">
-        <v>431</v>
-      </c>
-      <c r="AE40" s="1" t="s">
-        <v>431</v>
-      </c>
-      <c r="AF40" s="1" t="s">
-        <v>431</v>
-      </c>
-    </row>
-    <row r="41" spans="1:32" x14ac:dyDescent="0.25">
-      <c r="A41" t="s">
-        <v>391</v>
-      </c>
-      <c r="B41" s="1">
-        <f t="shared" si="0"/>
-        <v>30</v>
-      </c>
-    </row>
-    <row r="42" spans="1:32" x14ac:dyDescent="0.25">
-      <c r="A42" t="s">
-        <v>392</v>
-      </c>
-      <c r="B42" s="1">
-        <f t="shared" si="0"/>
-        <v>30</v>
-      </c>
-    </row>
-    <row r="43" spans="1:32" x14ac:dyDescent="0.25">
-      <c r="A43" t="s">
-        <v>394</v>
-      </c>
-      <c r="B43" s="1">
-        <f t="shared" si="0"/>
-        <v>30</v>
-      </c>
-    </row>
-    <row r="44" spans="1:32" x14ac:dyDescent="0.25">
-      <c r="A44" t="s">
-        <v>381</v>
-      </c>
-      <c r="B44" s="1">
-        <f t="shared" si="0"/>
-        <v>28</v>
-      </c>
-      <c r="S44" s="1" t="s">
+      <c r="T26" s="1" t="s">
         <v>398</v>
       </c>
-      <c r="T44" s="1" t="s">
+      <c r="Z26" s="1" t="s">
         <v>398</v>
       </c>
-    </row>
-    <row r="45" spans="1:32" x14ac:dyDescent="0.25">
-      <c r="A45" t="s">
-        <v>281</v>
-      </c>
-      <c r="B45" s="1">
-        <f t="shared" si="0"/>
-        <v>25</v>
-      </c>
-      <c r="H45" s="1" t="s">
+      <c r="AF26" s="1" t="s">
         <v>398</v>
       </c>
-      <c r="N45" s="1" t="s">
-        <v>398</v>
-      </c>
-      <c r="T45" s="1" t="s">
-        <v>398</v>
-      </c>
-      <c r="Z45" s="1" t="s">
-        <v>398</v>
-      </c>
-      <c r="AF45" s="1" t="s">
-        <v>398</v>
-      </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:AF52" xr:uid="{59A23CC3-1A6A-46FD-BA52-7A9B0C051B2C}">
-    <sortState xmlns:xlrd2="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata2" ref="A2:AF52">
-      <sortCondition ref="A1:A52"/>
-    </sortState>
-  </autoFilter>
   <phoneticPr fontId="1" type="noConversion"/>
   <pageMargins left="0.511811024" right="0.511811024" top="0.78740157499999996" bottom="0.78740157499999996" header="0.31496062000000002" footer="0.31496062000000002"/>
 </worksheet>
@@ -7538,7 +7336,7 @@
         <v>129</v>
       </c>
     </row>
-    <row r="4" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:9" hidden="1" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
         <v>402</v>
       </c>
@@ -7567,7 +7365,7 @@
         <v>129</v>
       </c>
     </row>
-    <row r="5" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:9" hidden="1" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
         <v>261</v>
       </c>
@@ -7654,7 +7452,7 @@
         <v>129</v>
       </c>
     </row>
-    <row r="8" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="8" spans="1:9" hidden="1" x14ac:dyDescent="0.25">
       <c r="A8" t="s">
         <v>264</v>
       </c>
@@ -7741,7 +7539,7 @@
         <v>129</v>
       </c>
     </row>
-    <row r="11" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="11" spans="1:9" hidden="1" x14ac:dyDescent="0.25">
       <c r="A11" t="s">
         <v>404</v>
       </c>
@@ -7915,7 +7713,7 @@
         <v>129</v>
       </c>
     </row>
-    <row r="17" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="17" spans="1:9" hidden="1" x14ac:dyDescent="0.25">
       <c r="A17" t="s">
         <v>272</v>
       </c>
@@ -7944,7 +7742,7 @@
         <v>129</v>
       </c>
     </row>
-    <row r="18" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="18" spans="1:9" hidden="1" x14ac:dyDescent="0.25">
       <c r="A18" t="s">
         <v>273</v>
       </c>
@@ -8031,7 +7829,7 @@
         <v>129</v>
       </c>
     </row>
-    <row r="21" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="21" spans="1:9" hidden="1" x14ac:dyDescent="0.25">
       <c r="A21" t="s">
         <v>276</v>
       </c>
@@ -8111,8 +7909,8 @@
       <c r="G23" s="1">
         <v>8</v>
       </c>
-      <c r="H23" s="1">
-        <v>4</v>
+      <c r="H23" s="2">
+        <v>5</v>
       </c>
       <c r="I23" s="1" t="s">
         <v>129</v>
@@ -8321,7 +8119,7 @@
         <v>129</v>
       </c>
     </row>
-    <row r="31" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="31" spans="1:9" hidden="1" x14ac:dyDescent="0.25">
       <c r="A31" t="s">
         <v>285</v>
       </c>
@@ -8350,7 +8148,7 @@
         <v>129</v>
       </c>
     </row>
-    <row r="32" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="32" spans="1:9" hidden="1" x14ac:dyDescent="0.25">
       <c r="A32" t="s">
         <v>286</v>
       </c>
@@ -8430,8 +8228,8 @@
       <c r="G34" s="1">
         <v>8</v>
       </c>
-      <c r="H34" s="1">
-        <v>4</v>
+      <c r="H34" s="2">
+        <v>5</v>
       </c>
       <c r="I34" s="1" t="s">
         <v>129</v>
@@ -8582,7 +8380,7 @@
         <v>129</v>
       </c>
     </row>
-    <row r="40" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="40" spans="1:9" hidden="1" x14ac:dyDescent="0.25">
       <c r="A40" t="s">
         <v>297</v>
       </c>
@@ -8952,8 +8750,8 @@
       <c r="G52" s="1">
         <v>8</v>
       </c>
-      <c r="H52" s="1">
-        <v>4</v>
+      <c r="H52" s="2">
+        <v>5</v>
       </c>
       <c r="I52" s="1" t="s">
         <v>129</v>
@@ -9046,7 +8844,7 @@
         <v>129</v>
       </c>
     </row>
-    <row r="56" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="56" spans="1:9" hidden="1" x14ac:dyDescent="0.25">
       <c r="A56" t="s">
         <v>311</v>
       </c>
@@ -9162,7 +8960,7 @@
         <v>129</v>
       </c>
     </row>
-    <row r="60" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="60" spans="1:9" hidden="1" x14ac:dyDescent="0.25">
       <c r="A60" t="s">
         <v>409</v>
       </c>
@@ -9213,8 +9011,8 @@
       <c r="G61" s="1">
         <v>8</v>
       </c>
-      <c r="H61" s="1">
-        <v>4</v>
+      <c r="H61" s="2">
+        <v>5</v>
       </c>
       <c r="I61" s="1" t="s">
         <v>129</v>
@@ -9481,7 +9279,7 @@
         <v>129</v>
       </c>
     </row>
-    <row r="71" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="71" spans="1:9" hidden="1" x14ac:dyDescent="0.25">
       <c r="A71" t="s">
         <v>410</v>
       </c>
@@ -9510,7 +9308,7 @@
         <v>129</v>
       </c>
     </row>
-    <row r="72" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="72" spans="1:9" hidden="1" x14ac:dyDescent="0.25">
       <c r="A72" t="s">
         <v>326</v>
       </c>
@@ -9568,7 +9366,7 @@
         <v>129</v>
       </c>
     </row>
-    <row r="74" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="74" spans="1:9" hidden="1" x14ac:dyDescent="0.25">
       <c r="A74" t="s">
         <v>411</v>
       </c>
@@ -9626,7 +9424,7 @@
         <v>129</v>
       </c>
     </row>
-    <row r="76" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="76" spans="1:9" hidden="1" x14ac:dyDescent="0.25">
       <c r="A76" t="s">
         <v>329</v>
       </c>
@@ -9684,7 +9482,7 @@
         <v>129</v>
       </c>
     </row>
-    <row r="78" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="78" spans="1:9" hidden="1" x14ac:dyDescent="0.25">
       <c r="A78" t="s">
         <v>331</v>
       </c>
@@ -9713,7 +9511,7 @@
         <v>129</v>
       </c>
     </row>
-    <row r="79" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="79" spans="1:9" hidden="1" x14ac:dyDescent="0.25">
       <c r="A79" t="s">
         <v>412</v>
       </c>
@@ -9771,7 +9569,7 @@
         <v>129</v>
       </c>
     </row>
-    <row r="81" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="81" spans="1:9" hidden="1" x14ac:dyDescent="0.25">
       <c r="A81" t="s">
         <v>334</v>
       </c>
@@ -9858,7 +9656,7 @@
         <v>129</v>
       </c>
     </row>
-    <row r="84" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="84" spans="1:9" hidden="1" x14ac:dyDescent="0.25">
       <c r="A84" t="s">
         <v>336</v>
       </c>
@@ -10467,7 +10265,7 @@
         <v>129</v>
       </c>
     </row>
-    <row r="105" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="105" spans="1:9" hidden="1" x14ac:dyDescent="0.25">
       <c r="A105" t="s">
         <v>415</v>
       </c>
@@ -10670,7 +10468,7 @@
         <v>129</v>
       </c>
     </row>
-    <row r="112" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="112" spans="1:9" hidden="1" x14ac:dyDescent="0.25">
       <c r="A112" t="s">
         <v>435</v>
       </c>
@@ -10699,7 +10497,7 @@
         <v>129</v>
       </c>
     </row>
-    <row r="113" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="113" spans="1:9" hidden="1" x14ac:dyDescent="0.25">
       <c r="A113" t="s">
         <v>436</v>
       </c>
@@ -10728,7 +10526,7 @@
         <v>129</v>
       </c>
     </row>
-    <row r="114" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="114" spans="1:9" hidden="1" x14ac:dyDescent="0.25">
       <c r="A114" t="s">
         <v>420</v>
       </c>
@@ -10757,7 +10555,7 @@
         <v>129</v>
       </c>
     </row>
-    <row r="115" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="115" spans="1:9" hidden="1" x14ac:dyDescent="0.25">
       <c r="A115" t="s">
         <v>418</v>
       </c>
@@ -10786,7 +10584,7 @@
         <v>129</v>
       </c>
     </row>
-    <row r="116" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="116" spans="1:9" hidden="1" x14ac:dyDescent="0.25">
       <c r="A116" t="s">
         <v>433</v>
       </c>
@@ -10815,7 +10613,7 @@
         <v>129</v>
       </c>
     </row>
-    <row r="117" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="117" spans="1:9" hidden="1" x14ac:dyDescent="0.25">
       <c r="A117" t="s">
         <v>434</v>
       </c>
@@ -10844,7 +10642,7 @@
         <v>129</v>
       </c>
     </row>
-    <row r="118" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="118" spans="1:9" hidden="1" x14ac:dyDescent="0.25">
       <c r="A118" t="s">
         <v>419</v>
       </c>
@@ -10873,7 +10671,7 @@
         <v>129</v>
       </c>
     </row>
-    <row r="119" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="119" spans="1:9" hidden="1" x14ac:dyDescent="0.25">
       <c r="A119" t="s">
         <v>365</v>
       </c>
@@ -10989,7 +10787,7 @@
         <v>129</v>
       </c>
     </row>
-    <row r="123" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="123" spans="1:9" hidden="1" x14ac:dyDescent="0.25">
       <c r="A123" t="s">
         <v>360</v>
       </c>
@@ -11018,7 +10816,7 @@
         <v>129</v>
       </c>
     </row>
-    <row r="124" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="124" spans="1:9" hidden="1" x14ac:dyDescent="0.25">
       <c r="A124" t="s">
         <v>361</v>
       </c>
@@ -11047,7 +10845,7 @@
         <v>129</v>
       </c>
     </row>
-    <row r="125" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="125" spans="1:9" hidden="1" x14ac:dyDescent="0.25">
       <c r="A125" t="s">
         <v>362</v>
       </c>
@@ -11163,7 +10961,7 @@
         <v>129</v>
       </c>
     </row>
-    <row r="129" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="129" spans="1:9" hidden="1" x14ac:dyDescent="0.25">
       <c r="A129" t="s">
         <v>367</v>
       </c>
@@ -11279,7 +11077,7 @@
         <v>129</v>
       </c>
     </row>
-    <row r="133" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="133" spans="1:9" hidden="1" x14ac:dyDescent="0.25">
       <c r="A133" t="s">
         <v>371</v>
       </c>
@@ -11388,8 +11186,8 @@
       <c r="G136" s="1">
         <v>8</v>
       </c>
-      <c r="H136" s="1">
-        <v>4</v>
+      <c r="H136" s="2">
+        <v>5</v>
       </c>
       <c r="I136" s="1" t="s">
         <v>129</v>
@@ -11743,7 +11541,7 @@
         <v>129</v>
       </c>
     </row>
-    <row r="149" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="149" spans="1:9" hidden="1" x14ac:dyDescent="0.25">
       <c r="A149" t="s">
         <v>388</v>
       </c>
@@ -11772,7 +11570,7 @@
         <v>129</v>
       </c>
     </row>
-    <row r="150" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="150" spans="1:9" hidden="1" x14ac:dyDescent="0.25">
       <c r="A150" t="s">
         <v>386</v>
       </c>
@@ -11830,7 +11628,7 @@
         <v>129</v>
       </c>
     </row>
-    <row r="152" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="152" spans="1:9" hidden="1" x14ac:dyDescent="0.25">
       <c r="A152" t="s">
         <v>389</v>
       </c>
@@ -12004,7 +11802,7 @@
         <v>129</v>
       </c>
     </row>
-    <row r="158" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="158" spans="1:9" hidden="1" x14ac:dyDescent="0.25">
       <c r="A158" t="s">
         <v>393</v>
       </c>
@@ -12033,7 +11831,7 @@
         <v>129</v>
       </c>
     </row>
-    <row r="159" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="159" spans="1:9" hidden="1" x14ac:dyDescent="0.25">
       <c r="A159" t="s">
         <v>394</v>
       </c>
@@ -12062,7 +11860,7 @@
         <v>129</v>
       </c>
     </row>
-    <row r="160" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="160" spans="1:9" hidden="1" x14ac:dyDescent="0.25">
       <c r="A160" t="s">
         <v>395</v>
       </c>
@@ -14003,6 +13801,15 @@
     </row>
   </sheetData>
   <autoFilter ref="A1:I161" xr:uid="{00000000-0001-0000-0100-000000000000}">
+    <filterColumn colId="0">
+      <filters>
+        <filter val="CAIQUE"/>
+        <filter val="DANILO"/>
+        <filter val="GISLENE"/>
+        <filter val="JAQUELINE FREITAS"/>
+        <filter val="SILAS"/>
+      </filters>
+    </filterColumn>
     <filterColumn colId="7">
       <filters>
         <filter val="4"/>

</xml_diff>